<commit_message>
#2 Routing completed BOM and Deliverables generated too
</commit_message>
<xml_diff>
--- a/Design-Files/AudioMoth-v1.2.0/BOM/JLCPCB-BOM-AudioMoth-v1.2.0.xlsx
+++ b/Design-Files/AudioMoth-v1.2.0/BOM/JLCPCB-BOM-AudioMoth-v1.2.0.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="141">
   <si>
     <t>Comment</t>
   </si>
@@ -176,18 +176,6 @@
     <t>C44838</t>
   </si>
   <si>
-    <t>DNP</t>
-  </si>
-  <si>
-    <t>J2</t>
-  </si>
-  <si>
-    <t>HDR1X2_</t>
-  </si>
-  <si>
-    <t>C706874</t>
-  </si>
-  <si>
     <t>1050170001</t>
   </si>
   <si>
@@ -197,15 +185,6 @@
     <t>C136000</t>
   </si>
   <si>
-    <t>J4</t>
-  </si>
-  <si>
-    <t>HDR1X3_</t>
-  </si>
-  <si>
-    <t>C706875</t>
-  </si>
-  <si>
     <t>693071010811</t>
   </si>
   <si>
@@ -293,9 +272,6 @@
     <t>C60490</t>
   </si>
   <si>
-    <t>R2</t>
-  </si>
-  <si>
     <t>15R</t>
   </si>
   <si>
@@ -324,9 +300,6 @@
   </si>
   <si>
     <t>C106231</t>
-  </si>
-  <si>
-    <t>R8, R13</t>
   </si>
   <si>
     <t>1R</t>
@@ -1190,7 +1163,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1212,15 +1185,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1566,7 +1530,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:D80"/>
+  <dimension ref="A1:D76"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="18.7142857142857" style="2" customWidth="1"/>
@@ -1590,55 +1554,55 @@
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="12" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="D3" s="14" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="14" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="14" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="8" t="s">
@@ -1646,770 +1610,714 @@
       </c>
     </row>
     <row r="6" spans="1:4">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="14" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:4">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="14" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:4">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="17" t="s">
+      <c r="D8" s="14" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:4">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="17" t="s">
+      <c r="D9" s="14" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:4">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="D10" s="17" t="s">
+      <c r="D10" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:4">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="14" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:4">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="17" t="s">
+      <c r="D12" s="14" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:4">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="14" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:4">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="C14" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="D14" s="17" t="s">
+      <c r="D14" s="14" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:4">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="C15" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D15" s="17" t="s">
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="13" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="16" t="s">
+      <c r="B16" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="C16" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="D16" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="C16" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="D16" s="17" t="s">
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="13" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="C17" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="D17" s="17" t="s">
+      <c r="D17" s="14" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:4">
-      <c r="A18" s="16" t="s">
+      <c r="A18" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="D18" s="17" t="s">
+      <c r="C18" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D18" s="14" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:4">
-      <c r="A19" s="16" t="s">
+      <c r="A19" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="C19" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="D19" s="17" t="s">
+      <c r="D19" s="14" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="20" spans="1:4">
-      <c r="A20" s="16" t="s">
+      <c r="A20" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="C20" s="17" t="s">
-        <v>64</v>
-      </c>
-      <c r="D20" s="17" t="s">
+      <c r="C20" s="14" t="s">
         <v>68</v>
       </c>
+      <c r="D20" s="14" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="21" spans="1:4">
-      <c r="A21" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="B21" s="17" t="s">
+      <c r="A21" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="C21" s="17" t="s">
+      <c r="B21" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="D21" s="17" t="s">
+      <c r="C21" s="14" t="s">
         <v>72</v>
       </c>
+      <c r="D21" s="14" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="22" spans="1:4">
-      <c r="A22" s="16" t="s">
-        <v>73</v>
-      </c>
-      <c r="B22" s="17" t="s">
+      <c r="A22" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="B22" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="D22" s="17" t="s">
+      <c r="C22" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="D22" s="14" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="23" spans="1:4">
-      <c r="A23" s="16" t="s">
+      <c r="A23" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="C23" s="17" t="s">
+      <c r="C23" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="D23" s="17" t="s">
+      <c r="D23" s="14" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="24" spans="1:4">
-      <c r="A24" s="16" t="s">
+      <c r="A24" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="C24" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="D24" s="17" t="s">
+      <c r="C24" s="14" t="s">
         <v>83</v>
       </c>
+      <c r="D24" s="14" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="25" spans="1:4">
-      <c r="A25" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="B25" s="17" t="s">
+      <c r="A25" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="C25" s="17" t="s">
+      <c r="B25" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="D25" s="17" t="s">
+      <c r="C25" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="D25" s="14" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="26" spans="1:4">
-      <c r="A26" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="B26" s="17" t="s">
+      <c r="A26" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="C26" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="D26" s="17" t="s">
-        <v>87</v>
+      <c r="B26" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="D26" s="14" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="27" spans="1:4">
-      <c r="A27" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="B27" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="C27" s="17" t="s">
+      <c r="A27" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="D27" s="17" t="s">
+      <c r="B27" s="14" t="s">
         <v>92</v>
       </c>
+      <c r="C27" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="D27" s="14" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="28" spans="1:4">
-      <c r="A28" s="16" t="s">
-        <v>93</v>
-      </c>
-      <c r="B28" s="17" t="s">
+      <c r="A28" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="B28" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="C28" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="D28" s="17" t="s">
+      <c r="C28" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="D28" s="14" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="29" spans="1:4">
-      <c r="A29" s="16" t="s">
+      <c r="A29" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="B29" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="C29" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="D29" s="17" t="s">
+      <c r="C29" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="D29" s="14" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="30" spans="1:4">
-      <c r="A30" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="B30" s="17" t="s">
+      <c r="A30" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="C30" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="D30" s="17" t="s">
-        <v>98</v>
+      <c r="B30" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="C30" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="31" spans="1:4">
-      <c r="A31" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="B31" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="C31" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="D31" s="17" t="s">
+      <c r="A31" s="13" t="s">
         <v>102</v>
       </c>
+      <c r="B31" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="32" spans="1:4">
-      <c r="A32" s="16" t="s">
-        <v>96</v>
-      </c>
-      <c r="B32" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="C32" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="D32" s="17" t="s">
-        <v>104</v>
+      <c r="A32" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="B32" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="D32" s="14" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="33" spans="1:4">
-      <c r="A33" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="B33" s="17" t="s">
-        <v>106</v>
-      </c>
-      <c r="C33" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="D33" s="17" t="s">
-        <v>107</v>
+      <c r="A33" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="B33" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="C33" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="34" spans="1:4">
-      <c r="A34" s="16" t="s">
-        <v>108</v>
-      </c>
-      <c r="B34" s="17" t="s">
-        <v>109</v>
-      </c>
-      <c r="C34" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="D34" s="17" t="s">
-        <v>110</v>
+      <c r="A34" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="B34" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="C34" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="D34" s="14" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="35" spans="1:4">
-      <c r="A35" s="16" t="s">
-        <v>111</v>
-      </c>
-      <c r="B35" s="17" t="s">
-        <v>112</v>
-      </c>
-      <c r="C35" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="D35" s="17" t="s">
-        <v>113</v>
+      <c r="A35" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="B35" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="C35" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="36" spans="1:4">
-      <c r="A36" s="16" t="s">
-        <v>114</v>
-      </c>
-      <c r="B36" s="17" t="s">
-        <v>115</v>
-      </c>
-      <c r="C36" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="D36" s="17" t="s">
-        <v>116</v>
+      <c r="A36" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="B36" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="37" spans="1:4">
-      <c r="A37" s="16" t="s">
-        <v>117</v>
-      </c>
-      <c r="B37" s="17" t="s">
-        <v>118</v>
-      </c>
-      <c r="C37" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="D37" s="17" t="s">
-        <v>119</v>
+      <c r="A37" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="B37" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="C37" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" s="16" t="s">
-        <v>120</v>
-      </c>
-      <c r="B38" s="17" t="s">
-        <v>121</v>
-      </c>
-      <c r="C38" s="17" t="s">
-        <v>120</v>
-      </c>
-      <c r="D38" s="17" t="s">
-        <v>122</v>
+      <c r="A38" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="B38" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="39" spans="1:4">
-      <c r="A39" s="16" t="s">
-        <v>123</v>
-      </c>
-      <c r="B39" s="17" t="s">
-        <v>124</v>
-      </c>
-      <c r="C39" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>126</v>
+      <c r="A39" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="B39" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="C39" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="D39" s="14" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="40" spans="1:4">
-      <c r="A40" s="16" t="s">
-        <v>127</v>
-      </c>
-      <c r="B40" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="C40" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="D40" s="8" t="s">
-        <v>130</v>
+      <c r="A40" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="B40" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="C40" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="D40" s="14" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="41" spans="1:4">
-      <c r="A41" s="16" t="s">
-        <v>131</v>
-      </c>
-      <c r="B41" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="C41" s="17" t="s">
-        <v>131</v>
-      </c>
-      <c r="D41" s="8" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4">
-      <c r="A42" s="16" t="s">
-        <v>134</v>
-      </c>
-      <c r="B42" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="C42" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="D42" s="17" t="s">
+      <c r="A41" s="14" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="43" spans="1:4">
-      <c r="A43" s="16" t="s">
+      <c r="B41" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="B43" s="17" t="s">
+      <c r="C41" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="C43" s="17" t="s">
+      <c r="D41" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="D43" s="17" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4">
-      <c r="A44" s="16" t="s">
-        <v>142</v>
-      </c>
-      <c r="B44" s="17" t="s">
-        <v>143</v>
-      </c>
-      <c r="C44" s="17" t="s">
-        <v>144</v>
-      </c>
-      <c r="D44" s="17" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4">
-      <c r="A45" s="17" t="s">
-        <v>146</v>
-      </c>
-      <c r="B45" s="17" t="s">
-        <v>147</v>
-      </c>
-      <c r="C45" s="17" t="s">
-        <v>148</v>
-      </c>
-      <c r="D45" s="17" t="s">
-        <v>149</v>
-      </c>
+    </row>
+    <row r="42" s="1" customFormat="1" spans="1:4">
+      <c r="A42" s="9"/>
+      <c r="B42" s="9"/>
+      <c r="C42" s="9"/>
+      <c r="D42" s="9"/>
+    </row>
+    <row r="43" s="1" customFormat="1" spans="1:4">
+      <c r="A43" s="9"/>
+      <c r="B43" s="9"/>
+      <c r="C43" s="9"/>
+      <c r="D43" s="9"/>
+    </row>
+    <row r="44" s="1" customFormat="1" spans="1:4">
+      <c r="A44" s="9"/>
+      <c r="B44" s="9"/>
+      <c r="C44" s="9"/>
+      <c r="D44" s="9"/>
+    </row>
+    <row r="45" s="1" customFormat="1" spans="1:4">
+      <c r="A45" s="9"/>
+      <c r="B45" s="9"/>
+      <c r="C45" s="9"/>
+      <c r="D45" s="9"/>
     </row>
     <row r="46" s="1" customFormat="1" spans="1:4">
       <c r="A46" s="9"/>
-      <c r="B46" s="10"/>
-      <c r="C46" s="10"/>
-      <c r="D46" s="10"/>
+      <c r="B46" s="9"/>
+      <c r="C46" s="9"/>
+      <c r="D46" s="9"/>
     </row>
     <row r="47" s="1" customFormat="1" spans="1:4">
       <c r="A47" s="9"/>
-      <c r="B47" s="10"/>
-      <c r="C47" s="10"/>
-      <c r="D47" s="10"/>
+      <c r="B47" s="9"/>
+      <c r="C47" s="9"/>
+      <c r="D47" s="9"/>
     </row>
     <row r="48" s="1" customFormat="1" spans="1:4">
       <c r="A48" s="9"/>
-      <c r="B48" s="10"/>
-      <c r="C48" s="10"/>
-      <c r="D48" s="10"/>
+      <c r="B48" s="9"/>
+      <c r="C48" s="9"/>
+      <c r="D48" s="9"/>
     </row>
     <row r="49" s="1" customFormat="1" spans="1:4">
       <c r="A49" s="9"/>
-      <c r="B49" s="10"/>
-      <c r="C49" s="10"/>
-      <c r="D49" s="10"/>
+      <c r="B49" s="9"/>
+      <c r="C49" s="9"/>
+      <c r="D49" s="9"/>
     </row>
     <row r="50" s="1" customFormat="1" spans="1:4">
       <c r="A50" s="9"/>
-      <c r="B50" s="10"/>
-      <c r="C50" s="10"/>
-      <c r="D50" s="10"/>
+      <c r="B50" s="9"/>
+      <c r="C50" s="9"/>
+      <c r="D50" s="9"/>
     </row>
     <row r="51" s="1" customFormat="1" spans="1:4">
       <c r="A51" s="9"/>
-      <c r="B51" s="10"/>
-      <c r="C51" s="10"/>
-      <c r="D51" s="10"/>
+      <c r="B51" s="9"/>
+      <c r="C51" s="9"/>
+      <c r="D51" s="9"/>
     </row>
     <row r="52" s="1" customFormat="1" spans="1:4">
       <c r="A52" s="9"/>
-      <c r="B52" s="10"/>
-      <c r="C52" s="10"/>
-      <c r="D52" s="10"/>
+      <c r="B52" s="9"/>
+      <c r="C52" s="9"/>
+      <c r="D52" s="9"/>
     </row>
     <row r="53" s="1" customFormat="1" spans="1:4">
       <c r="A53" s="9"/>
-      <c r="B53" s="10"/>
-      <c r="C53" s="10"/>
-      <c r="D53" s="10"/>
+      <c r="B53" s="9"/>
+      <c r="C53" s="9"/>
+      <c r="D53" s="9"/>
     </row>
     <row r="54" s="1" customFormat="1" spans="1:4">
       <c r="A54" s="9"/>
-      <c r="B54" s="10"/>
-      <c r="C54" s="10"/>
-      <c r="D54" s="10"/>
+      <c r="B54" s="9"/>
+      <c r="C54" s="9"/>
+      <c r="D54" s="9"/>
     </row>
     <row r="55" s="1" customFormat="1" spans="1:4">
       <c r="A55" s="9"/>
-      <c r="B55" s="10"/>
-      <c r="C55" s="10"/>
-      <c r="D55" s="10"/>
+      <c r="B55" s="9"/>
+      <c r="C55" s="9"/>
+      <c r="D55" s="9"/>
     </row>
     <row r="56" s="1" customFormat="1" spans="1:4">
       <c r="A56" s="9"/>
-      <c r="B56" s="10"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="10"/>
+      <c r="B56" s="9"/>
+      <c r="C56" s="9"/>
+      <c r="D56" s="9"/>
     </row>
     <row r="57" s="1" customFormat="1" spans="1:4">
       <c r="A57" s="9"/>
-      <c r="B57" s="10"/>
-      <c r="C57" s="10"/>
-      <c r="D57" s="10"/>
+      <c r="B57" s="9"/>
+      <c r="C57" s="9"/>
+      <c r="D57" s="9"/>
     </row>
     <row r="58" s="1" customFormat="1" spans="1:4">
       <c r="A58" s="9"/>
-      <c r="B58" s="10"/>
-      <c r="C58" s="10"/>
-      <c r="D58" s="10"/>
+      <c r="B58" s="9"/>
+      <c r="C58" s="9"/>
+      <c r="D58" s="9"/>
     </row>
     <row r="59" s="1" customFormat="1" spans="1:4">
       <c r="A59" s="9"/>
-      <c r="B59" s="10"/>
-      <c r="C59" s="10"/>
-      <c r="D59" s="10"/>
+      <c r="B59" s="9"/>
+      <c r="C59" s="9"/>
+      <c r="D59" s="9"/>
     </row>
     <row r="60" s="1" customFormat="1" spans="1:4">
       <c r="A60" s="9"/>
-      <c r="B60" s="10"/>
-      <c r="C60" s="10"/>
-      <c r="D60" s="10"/>
+      <c r="B60" s="9"/>
+      <c r="C60" s="9"/>
+      <c r="D60" s="9"/>
     </row>
     <row r="61" s="1" customFormat="1" spans="1:4">
       <c r="A61" s="9"/>
-      <c r="B61" s="10"/>
-      <c r="C61" s="10"/>
-      <c r="D61" s="10"/>
+      <c r="B61" s="9"/>
+      <c r="C61" s="9"/>
+      <c r="D61" s="9"/>
     </row>
     <row r="62" s="1" customFormat="1" spans="1:4">
       <c r="A62" s="9"/>
-      <c r="B62" s="10"/>
-      <c r="C62" s="10"/>
-      <c r="D62" s="10"/>
+      <c r="B62" s="9"/>
+      <c r="C62" s="9"/>
+      <c r="D62" s="9"/>
     </row>
     <row r="63" s="1" customFormat="1" spans="1:4">
       <c r="A63" s="9"/>
-      <c r="B63" s="10"/>
-      <c r="C63" s="10"/>
-      <c r="D63" s="10"/>
+      <c r="B63" s="9"/>
+      <c r="C63" s="9"/>
+      <c r="D63" s="9"/>
     </row>
     <row r="64" s="1" customFormat="1" spans="1:4">
       <c r="A64" s="9"/>
-      <c r="B64" s="10"/>
-      <c r="C64" s="10"/>
-      <c r="D64" s="10"/>
+      <c r="B64" s="9"/>
+      <c r="C64" s="9"/>
+      <c r="D64" s="9"/>
     </row>
     <row r="65" s="1" customFormat="1" spans="1:4">
       <c r="A65" s="9"/>
-      <c r="B65" s="10"/>
-      <c r="C65" s="10"/>
-      <c r="D65" s="10"/>
+      <c r="B65" s="9"/>
+      <c r="C65" s="9"/>
+      <c r="D65" s="9"/>
     </row>
     <row r="66" s="1" customFormat="1" spans="1:4">
       <c r="A66" s="9"/>
-      <c r="B66" s="10"/>
-      <c r="C66" s="10"/>
-      <c r="D66" s="10"/>
+      <c r="B66" s="9"/>
+      <c r="C66" s="9"/>
+      <c r="D66" s="9"/>
     </row>
     <row r="67" s="1" customFormat="1" spans="1:4">
       <c r="A67" s="9"/>
-      <c r="B67" s="10"/>
-      <c r="C67" s="10"/>
-      <c r="D67" s="10"/>
+      <c r="B67" s="9"/>
+      <c r="C67" s="9"/>
+      <c r="D67" s="9"/>
     </row>
     <row r="68" s="1" customFormat="1" spans="1:4">
       <c r="A68" s="9"/>
-      <c r="B68" s="10"/>
-      <c r="C68" s="10"/>
-      <c r="D68" s="10"/>
+      <c r="B68" s="9"/>
+      <c r="C68" s="9"/>
+      <c r="D68" s="9"/>
     </row>
     <row r="69" s="1" customFormat="1" spans="1:4">
       <c r="A69" s="9"/>
-      <c r="B69" s="10"/>
-      <c r="C69" s="10"/>
-      <c r="D69" s="10"/>
+      <c r="B69" s="9"/>
+      <c r="C69" s="9"/>
+      <c r="D69" s="9"/>
     </row>
     <row r="70" s="1" customFormat="1" spans="1:4">
       <c r="A70" s="9"/>
-      <c r="B70" s="10"/>
-      <c r="C70" s="10"/>
-      <c r="D70" s="10"/>
+      <c r="B70" s="9"/>
+      <c r="C70" s="9"/>
+      <c r="D70" s="9"/>
     </row>
     <row r="71" s="1" customFormat="1" spans="1:4">
       <c r="A71" s="9"/>
-      <c r="B71" s="10"/>
-      <c r="C71" s="10"/>
-      <c r="D71" s="10"/>
-    </row>
-    <row r="72" s="1" customFormat="1" spans="1:4">
-      <c r="A72" s="9"/>
-      <c r="B72" s="10"/>
-      <c r="C72" s="10"/>
-      <c r="D72" s="10"/>
+      <c r="B71" s="9"/>
+      <c r="C71" s="9"/>
+      <c r="D71" s="9"/>
+    </row>
+    <row r="72" s="1" customFormat="1" spans="2:4">
+      <c r="B72" s="9"/>
+      <c r="C72" s="9"/>
+      <c r="D72" s="9"/>
     </row>
     <row r="73" s="1" customFormat="1" spans="1:4">
       <c r="A73" s="9"/>
-      <c r="B73" s="10"/>
-      <c r="C73" s="10"/>
-      <c r="D73" s="10"/>
+      <c r="B73" s="9"/>
+      <c r="C73" s="9"/>
+      <c r="D73" s="9"/>
     </row>
     <row r="74" s="1" customFormat="1" spans="1:4">
       <c r="A74" s="9"/>
-      <c r="B74" s="10"/>
-      <c r="C74" s="10"/>
-      <c r="D74" s="10"/>
+      <c r="B74" s="9"/>
+      <c r="C74" s="9"/>
+      <c r="D74" s="9"/>
     </row>
     <row r="75" s="1" customFormat="1" spans="1:4">
       <c r="A75" s="9"/>
-      <c r="B75" s="10"/>
-      <c r="C75" s="10"/>
-      <c r="D75" s="10"/>
-    </row>
-    <row r="76" s="1" customFormat="1" spans="2:4">
-      <c r="B76" s="10"/>
-      <c r="C76" s="10"/>
-      <c r="D76" s="10"/>
-    </row>
-    <row r="77" s="1" customFormat="1" spans="1:4">
-      <c r="A77" s="9"/>
-      <c r="B77" s="10"/>
-      <c r="C77" s="10"/>
-      <c r="D77" s="10"/>
-    </row>
-    <row r="78" s="1" customFormat="1" spans="1:4">
-      <c r="A78" s="9"/>
-      <c r="B78" s="10"/>
-      <c r="C78" s="10"/>
-      <c r="D78" s="10"/>
-    </row>
-    <row r="79" s="1" customFormat="1" spans="1:4">
-      <c r="A79" s="11"/>
-      <c r="B79" s="12"/>
-      <c r="C79" s="12"/>
-      <c r="D79" s="12"/>
-    </row>
-    <row r="80" s="1" customFormat="1" spans="1:1">
-      <c r="A80" s="13"/>
+      <c r="B75" s="9"/>
+      <c r="C75" s="9"/>
+      <c r="D75" s="9"/>
+    </row>
+    <row r="76" s="1" customFormat="1" spans="1:1">
+      <c r="A76" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>